<commit_message>
docs: Refresh enchant DBC sheet from source
</commit_message>
<xml_diff>
--- a/강화DBC_시각화.xlsx
+++ b/강화DBC_시각화.xlsx
@@ -10,7 +10,7 @@
     <sheet name="강화DBC" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'강화DBC'!$A$1:$J$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'강화DBC'!$A$1:$K$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,19 +447,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,7 +511,12 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>DBC 설명</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>변경여부</t>
         </is>
       </c>
     </row>
@@ -544,7 +550,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
@@ -552,7 +558,12 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>힘 2 / 민첩 2 / 방관 1</t>
+          <t>힘 2 / 민첩 2 / 방어구 관통 1</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -597,6 +608,11 @@
           <t>주문력 1 / 지능 2 / 가속 1</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -639,6 +655,11 @@
           <t>지능 2 / 정신 1 / 가속 1</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -670,7 +691,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -678,7 +699,12 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>힘 1 / 체력 2 / 방숙 1</t>
+          <t>힘 1 / 체력 2 / 방어 숙련 1</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -712,7 +738,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -720,7 +746,12 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>힘 3 / 민첩 3 / 방관 2</t>
+          <t>힘 3 / 민첩 3 / 방어구 관통 2</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -765,6 +796,11 @@
           <t>주문력 2 / 지능 3 / 가속 2</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -807,6 +843,11 @@
           <t>지능 3 / 정신 2 / 가속 2</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -838,7 +879,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
@@ -846,7 +887,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>힘 3 / 체력 4 / 방숙 2</t>
+          <t>힘 3 / 체력 4 / 방어 숙련 2</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -880,7 +926,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -888,7 +934,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>힘 4 / 민첩 4 / 방관 3</t>
+          <t>힘 4 / 민첩 4 / 방어구 관통 3</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -933,6 +984,11 @@
           <t>주문력 3 / 지능 4 / 가속 3</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -975,6 +1031,11 @@
           <t>지능 4 / 정신 3 / 가속 3</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1006,7 +1067,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
@@ -1014,7 +1075,12 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>힘 4 / 체력 5 / 방숙 2</t>
+          <t>힘 4 / 체력 5 / 방어 숙련 2</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1114,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
@@ -1056,7 +1122,12 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>힘 5 / 민첩 5 / 방관 4</t>
+          <t>힘 5 / 민첩 5 / 방어구 관통 4</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1101,6 +1172,11 @@
           <t>주문력 4 / 지능 5 / 가속 4</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1143,6 +1219,11 @@
           <t>지능 5 / 정신 4 / 가속 4</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1174,7 +1255,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I17" s="2" t="n">
@@ -1182,7 +1263,12 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>힘 5 / 체력 6 / 방숙 3</t>
+          <t>힘 5 / 체력 6 / 방어 숙련 3</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1302,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I18" s="2" t="n">
@@ -1224,7 +1310,12 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>힘 7 / 민첩 7 / 방관 5</t>
+          <t>힘 7 / 민첩 7 / 방어구 관통 5</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1269,6 +1360,11 @@
           <t>주문력 5 / 지능 6 / 가속 5</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1311,6 +1407,11 @@
           <t>지능 6 / 정신 6 / 가속 5</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1342,7 +1443,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
@@ -1350,7 +1451,12 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>힘 7 / 체력 7 / 방숙 3</t>
+          <t>힘 7 / 체력 7 / 방어 숙련 3</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1490,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
@@ -1392,7 +1498,12 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>힘 8 / 민첩 8 / 방관 6</t>
+          <t>힘 8 / 민첩 8 / 방어구 관통 6</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1437,6 +1548,11 @@
           <t>주문력 7 / 지능 8 / 가속 7</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1479,6 +1595,11 @@
           <t>지능 8 / 정신 7 / 가속 7</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1510,7 +1631,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I25" s="2" t="n">
@@ -1518,7 +1639,12 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>힘 8 / 체력 9 / 방숙 4</t>
+          <t>힘 8 / 체력 9 / 방어 숙련 4</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1678,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
@@ -1560,7 +1686,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>힘 9 / 민첩 9 / 방관 7</t>
+          <t>힘 9 / 민첩 9 / 방어구 관통 7</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1605,6 +1736,11 @@
           <t>주문력 8 / 지능 9 / 가속 8</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1647,6 +1783,11 @@
           <t>지능 10 / 정신 9 / 가속 8</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1678,7 +1819,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
@@ -1686,7 +1827,12 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>힘 9 / 체력 10 / 방숙 4</t>
+          <t>힘 9 / 체력 10 / 방어 숙련 4</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1866,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
@@ -1728,7 +1874,12 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>힘 11 / 민첩 11 / 방관 8</t>
+          <t>힘 11 / 민첩 11 / 방어구 관통 8</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1773,6 +1924,11 @@
           <t>주문력 9 / 지능 11 / 가속 9</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1815,6 +1971,11 @@
           <t>지능 12 / 정신 10 / 가속 10</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1846,7 +2007,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -1854,7 +2015,12 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>힘 11 / 체력 12 / 방숙 5</t>
+          <t>힘 11 / 체력 12 / 방어 숙련 5</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1888,7 +2054,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
@@ -1896,7 +2062,12 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>힘 12 / 민첩 12 / 방관 9</t>
+          <t>힘 12 / 민첩 12 / 방어구 관통 9</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1941,6 +2112,11 @@
           <t>주문력 11 / 지능 13 / 가속 11</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1983,6 +2159,11 @@
           <t>지능 13 / 정신 12 / 가속 11</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2014,7 +2195,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
@@ -2022,7 +2203,12 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>힘 12 / 체력 13 / 방숙 5</t>
+          <t>힘 12 / 체력 13 / 방어 숙련 5</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2242,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>방관</t>
+          <t>방어구 관통</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
@@ -2064,7 +2250,12 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>힘 13 / 민첩 13 / 방관 10</t>
+          <t>힘 13 / 민첩 13 / 방어구 관통 10</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2109,6 +2300,11 @@
           <t>주문력 12 / 지능 15 / 가속 12</t>
         </is>
       </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2151,6 +2347,11 @@
           <t>지능 15 / 정신 15 / 가속 12</t>
         </is>
       </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2182,7 +2383,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>방숙</t>
+          <t>방어 숙련</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -2190,12 +2391,17 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>힘 13 / 체력 15 / 방숙 5</t>
+          <t>힘 13 / 체력 15 / 방어 숙련 5</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J41"/>
+  <autoFilter ref="A1:K41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>